<commit_message>
fix(historical-import): align synthetic fixtures with parser contract
</commit_message>
<xml_diff>
--- a/fixtures/historical-import/synthetic-survey-base.xlsx
+++ b/fixtures/historical-import/synthetic-survey-base.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="162">
   <si>
     <t>response_id</t>
   </si>
@@ -449,6 +449,24 @@
   </si>
   <si>
     <t>ROOT</t>
+  </si>
+  <si>
+    <t>H-DEP-SYN</t>
+  </si>
+  <si>
+    <t>Departamento Sintético</t>
+  </si>
+  <si>
+    <t>DEPARTMENT</t>
+  </si>
+  <si>
+    <t>H-AREA-SYN</t>
+  </si>
+  <si>
+    <t>Área Sintética</t>
+  </si>
+  <si>
+    <t>AREA</t>
   </si>
   <si>
     <t>H-DIV-DIV-A</t>
@@ -4387,7 +4405,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -4444,7 +4462,7 @@
         <v>142</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -4455,19 +4473,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D4" t="s">
         <v>145</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -4478,19 +4496,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C5" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D5" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -4501,19 +4519,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="D6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E6" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -4524,19 +4542,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C7" t="s">
         <v>153</v>
       </c>
-      <c r="B7" t="s">
-        <v>154</v>
-      </c>
-      <c r="C7" t="s">
-        <v>147</v>
-      </c>
       <c r="D7" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="E7" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -4547,25 +4565,71 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C8" t="s">
         <v>155</v>
       </c>
-      <c r="C8" t="s">
-        <v>149</v>
-      </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E8" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8">
         <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D9" t="s">
+        <v>148</v>
+      </c>
+      <c r="E9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" t="s">
+        <v>159</v>
+      </c>
+      <c r="E10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>